<commit_message>
feat(schema): render the Collections Ontology 2.0 with CO's names and IRIs
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/collections.xlsx
+++ b/project/excel/collections.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bag" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Collection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CoItem" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Collection" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Set" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bag" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="List" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ListItem" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Set" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CoItem" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ListItem" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,12 +424,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>co_size</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>element</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>size</t>
         </is>
       </c>
     </row>
@@ -450,12 +450,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>co_size</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>element</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>size</t>
         </is>
       </c>
     </row>
@@ -470,13 +470,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>itemOf</t>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>co_size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>element</t>
         </is>
       </c>
     </row>
@@ -497,27 +507,27 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>firstItem</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>lastItem</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>lastItem</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>firstItem</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>co_size</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>element</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>size</t>
         </is>
       </c>
     </row>
@@ -532,18 +542,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>_index</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>itemOf</t>
+          <t>itemContent</t>
         </is>
       </c>
     </row>
@@ -558,18 +563,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>size</t>
+          <t>nextItem</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>previousItem</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>followedBy</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>precededBy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>itemContent</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(schema): map CO's alignment, add CoElement and state more CO axioms
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/collections.xlsx
+++ b/project/excel/collections.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Set" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Bag" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="List" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CoItem" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ListItem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CoElement" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CoItem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ListItem" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -548,7 +549,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>itemContent</t>
+          <t>iri</t>
         </is>
       </c>
     </row>
@@ -558,6 +559,27 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>itemContent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(schema): map CO's alignment, add CoElement and state more CO axioms (#5)
* feat(schema): map CO's alignment, add CoElement and state more CO axioms

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* docs(lokf): link glossary terms to the schema and each other, add element

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* docs(schema): say monotonic inheritance keeps firstItem off item; cite #3950

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

* docs(lokf): give monotonic inheritance as the reason in scope-and-rules

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>

---------

Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/collections.xlsx
+++ b/project/excel/collections.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Set" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Bag" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="List" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CoItem" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ListItem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CoElement" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CoItem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ListItem" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -548,7 +549,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>itemContent</t>
+          <t>iri</t>
         </is>
       </c>
     </row>
@@ -558,6 +559,27 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>itemContent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>